<commit_message>
QA heat: workbook Model!B13 spark-ratio threshold read 13.42; energy-basis parity is eta_e/eta_g = 1.153
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/heat/lcoh_model.xlsx
+++ b/heat/lcoh_model.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Model" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sensitivity" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -933,11 +933,11 @@
     <row r="13" ht="15" customHeight="1" s="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Spark ratio threshold Pe/Pg (kWh-basis parity)</t>
+          <t>Spark ratio threshold, energy basis (= eta_e/eta_g)</t>
         </is>
       </c>
       <c r="B13" s="16">
-        <f>B12/Inputs!$B$7*1000000/Inputs!$B$17</f>
+        <f>B12*Inputs!$B$17/Inputs!$B$7</f>
         <v/>
       </c>
       <c r="C13" s="16" t="n"/>

</xml_diff>